<commit_message>
Pair export-list batches on the declared value too, not only the anchor
The export list quotes the value declared on the tranche sheet. For a
re-tested batch that is not our latest verified result, so pairing on the
anchor alone made five re-tested batches look as though they had no
certificate at all. All 77 now resolve; the five had certificates all along,
and two of them carry a newer result that changes the export class.
</commit_message>
<xml_diff>
--- a/deliverables/potency_study/Potency_Specs_and_Results.xlsx
+++ b/deliverables/potency_study/Potency_Specs_and_Results.xlsx
@@ -440,10 +440,10 @@
     <xf numFmtId="0" fontId="28" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -10657,7 +10657,7 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>KC102501</t>
         </is>
       </c>
       <c r="G46" s="26" t="inlineStr">
@@ -10667,22 +10667,22 @@
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I46" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J46" s="49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K46" s="28" t="inlineStr">
-        <is>
-          <t>нема декларирана класа | no declared grade</t>
+          <t>17.04%</t>
+        </is>
+      </c>
+      <c r="I46" s="48" t="inlineStr">
+        <is>
+          <t>-0.36</t>
+        </is>
+      </c>
+      <c r="J46" s="13" t="inlineStr">
+        <is>
+          <t>Pot.-1</t>
+        </is>
+      </c>
+      <c r="K46" s="40" t="inlineStr">
+        <is>
+          <t>17.00% ± 1.70% (15.30%–18.70%)</t>
         </is>
       </c>
       <c r="L46" s="41" t="n">
@@ -10698,17 +10698,15 @@
           <t>19.80</t>
         </is>
       </c>
-      <c r="O46" s="50" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="O46" s="29" t="n">
+        <v>18</v>
       </c>
       <c r="P46" s="26" t="n">
         <v>16</v>
       </c>
       <c r="Q46" s="43" t="inlineStr">
         <is>
-          <t>нема во регистарот/Атласот | not in register/Atlas</t>
+          <t>серијата е спарена по доказ (сорта + вредност) | batch paired by evidence; листата: 17.40% ≠ наш: 17.04% | list vs ours</t>
         </is>
       </c>
     </row>
@@ -11038,7 +11036,7 @@
       </c>
       <c r="F51" s="17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PM112501</t>
         </is>
       </c>
       <c r="G51" s="24" t="inlineStr">
@@ -11048,22 +11046,22 @@
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I51" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J51" s="49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K51" s="28" t="inlineStr">
-        <is>
-          <t>нема декларирана класа | no declared grade</t>
+          <t>13.33%</t>
+        </is>
+      </c>
+      <c r="I51" s="46" t="inlineStr">
+        <is>
+          <t>+0.33</t>
+        </is>
+      </c>
+      <c r="J51" s="13" t="inlineStr">
+        <is>
+          <t>Pot.-2</t>
+        </is>
+      </c>
+      <c r="K51" s="40" t="inlineStr">
+        <is>
+          <t>12.50% ± 1.25% (11.25%–13.75%)</t>
         </is>
       </c>
       <c r="L51" s="41" t="n">
@@ -11079,17 +11077,15 @@
           <t>15.40</t>
         </is>
       </c>
-      <c r="O51" s="50" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="O51" s="22" t="n">
+        <v>14</v>
       </c>
       <c r="P51" s="24" t="n">
         <v>48</v>
       </c>
       <c r="Q51" s="45" t="inlineStr">
         <is>
-          <t>нема во регистарот/Атласот | not in register/Atlas</t>
+          <t>серијата е спарена по доказ (сорта + вредност) | batch paired by evidence; листата: 13.00% ≠ наш: 13.33% | list vs ours</t>
         </is>
       </c>
     </row>
@@ -12399,7 +12395,7 @@
           <t>26.40</t>
         </is>
       </c>
-      <c r="O69" s="50" t="n">
+      <c r="O69" s="49" t="n">
         <v>26</v>
       </c>
       <c r="P69" s="26" t="n">
@@ -12553,7 +12549,7 @@
           <t>8.80</t>
         </is>
       </c>
-      <c r="O71" s="50" t="inlineStr">
+      <c r="O71" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -12672,7 +12668,7 @@
       </c>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>J31112501</t>
         </is>
       </c>
       <c r="G73" s="26" t="inlineStr">
@@ -12682,22 +12678,22 @@
       </c>
       <c r="H73" s="10" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I73" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J73" s="49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K73" s="28" t="inlineStr">
-        <is>
-          <t>нема декларирана класа | no declared grade</t>
+          <t>20.21%</t>
+        </is>
+      </c>
+      <c r="I73" s="48" t="inlineStr">
+        <is>
+          <t>-4.79</t>
+        </is>
+      </c>
+      <c r="J73" s="13" t="inlineStr">
+        <is>
+          <t>Pot.-2</t>
+        </is>
+      </c>
+      <c r="K73" s="40" t="inlineStr">
+        <is>
+          <t>21.00% ± 2.10% (18.90%–23.10%)</t>
         </is>
       </c>
       <c r="L73" s="41" t="n">
@@ -12713,17 +12709,15 @@
           <t>28.60</t>
         </is>
       </c>
-      <c r="O73" s="50" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="O73" s="49" t="n">
+        <v>22</v>
       </c>
       <c r="P73" s="26" t="n">
         <v>85.09999999999999</v>
       </c>
       <c r="Q73" s="43" t="inlineStr">
         <is>
-          <t>нема во регистарот/Атласот | not in register/Atlas</t>
+          <t>серијата е спарена по доказ (сорта + вредност) | batch paired by evidence; листата: 25.00% ≠ наш: 20.21% | list vs ours; по наш резултат: класа 22 | on our result: class 22</t>
         </is>
       </c>
     </row>
@@ -12753,7 +12747,7 @@
       </c>
       <c r="F74" s="17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>J31122501</t>
         </is>
       </c>
       <c r="G74" s="24" t="inlineStr">
@@ -12763,22 +12757,22 @@
       </c>
       <c r="H74" s="19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I74" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J74" s="49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K74" s="28" t="inlineStr">
-        <is>
-          <t>нема декларирана класа | no declared grade</t>
+          <t>21.84%</t>
+        </is>
+      </c>
+      <c r="I74" s="46" t="inlineStr">
+        <is>
+          <t>+0.07</t>
+        </is>
+      </c>
+      <c r="J74" s="13" t="inlineStr">
+        <is>
+          <t>Pot.-2</t>
+        </is>
+      </c>
+      <c r="K74" s="40" t="inlineStr">
+        <is>
+          <t>21.00% ± 2.10% (18.90%–23.10%)</t>
         </is>
       </c>
       <c r="L74" s="41" t="n">
@@ -12794,17 +12788,15 @@
           <t>26.40</t>
         </is>
       </c>
-      <c r="O74" s="50" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="O74" s="22" t="n">
+        <v>24</v>
       </c>
       <c r="P74" s="24" t="n">
         <v>135.49</v>
       </c>
       <c r="Q74" s="45" t="inlineStr">
         <is>
-          <t>нема во регистарот/Атласот | not in register/Atlas</t>
+          <t>серијата е спарена по доказ (сорта + вредност) | batch paired by evidence; листата: 21.77% ≠ наш: 21.84% | list vs ours</t>
         </is>
       </c>
     </row>
@@ -13375,7 +13367,7 @@
       </c>
       <c r="F82" s="17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SJ112501</t>
         </is>
       </c>
       <c r="G82" s="24" t="inlineStr">
@@ -13385,22 +13377,22 @@
       </c>
       <c r="H82" s="19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I82" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J82" s="49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K82" s="28" t="inlineStr">
-        <is>
-          <t>нема декларирана класа | no declared grade</t>
+          <t>9.20%</t>
+        </is>
+      </c>
+      <c r="I82" s="46" t="inlineStr">
+        <is>
+          <t>+0.20</t>
+        </is>
+      </c>
+      <c r="J82" s="13" t="inlineStr">
+        <is>
+          <t>Pot.-1</t>
+        </is>
+      </c>
+      <c r="K82" s="40" t="inlineStr">
+        <is>
+          <t>9.00% ± 0.89% (8.11%–9.89%)</t>
         </is>
       </c>
       <c r="L82" s="41" t="n">
@@ -13416,17 +13408,15 @@
           <t>11.00</t>
         </is>
       </c>
-      <c r="O82" s="50" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="O82" s="22" t="n">
+        <v>10</v>
       </c>
       <c r="P82" s="24" t="n">
         <v>50.62</v>
       </c>
       <c r="Q82" s="45" t="inlineStr">
         <is>
-          <t>нема во регистарот/Атласот | not in register/Atlas</t>
+          <t>серијата е спарена по доказ (сорта + вредност) | batch paired by evidence; листата: 9.00% ≠ наш: 9.20% | list vs ours</t>
         </is>
       </c>
     </row>
@@ -13624,7 +13614,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="J85" s="49" t="inlineStr">
+      <c r="J85" s="50" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -13647,7 +13637,7 @@
           <t>24.20</t>
         </is>
       </c>
-      <c r="O85" s="50" t="inlineStr">
+      <c r="O85" s="49" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>